<commit_message>
last changes for thesis
</commit_message>
<xml_diff>
--- a/UV-Vis/Plots/Summary_Bandgaps.xlsx
+++ b/UV-Vis/Plots/Summary_Bandgaps.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,16 +432,11 @@
           <t>Gap (eV)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Error (eV)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sb200</t>
+          <t>CdS1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -450,16 +445,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.201084788396404</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.09594243273782281</v>
+        <v>2.238377246593132</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sb200</t>
+          <t>CdS1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -468,16 +460,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.112809405129241</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.05358192065359806</v>
+        <v>1.424397396537707</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sb300</t>
+          <t>CdS2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -486,16 +475,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.196451458058087</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.09106605469441002</v>
+        <v>2.126251268160163</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sb300</t>
+          <t>CdS2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -504,16 +490,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.104671720995331</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.05089960295758991</v>
+        <v>1.270211418526796</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sb400</t>
+          <t>CdS3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -522,16 +505,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.191277916771089</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.09102351330055976</v>
+        <v>1.962366367582087</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sb400</t>
+          <t>CdS3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -540,226 +520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.111695526525509</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.04921159029328564</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Mo_25Se_200Sb</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1.129801596051832</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.0412271176589978</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mo_25Se_200Sb</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Indirect</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.9860919956939599</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.0232035051469779</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mo_125Se_200Sb</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1.134629018804752</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.06335461504731341</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mo_125Se_200Sb</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Indirect</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0.8897474050259655</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.04254422120919129</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Mo_25Se_300Sb</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>1.170478039530471</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.06841814052637445</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mo_25Se_300Sb</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Indirect</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>0.9930569202440097</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.04308117309271923</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Mo_125Se_300Sb</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1.184143034864894</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.0780094018372882</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Mo_125Se_300Sb</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Indirect</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1.047598390089843</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.04900609120275409</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Mo_25Se_400Sb</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>1.180588721930234</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.07196233614548796</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Mo_25Se_400Sb</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Indirect</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>1.038327700222461</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.04238852094206078</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Mo_125Se_400Sb</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>1.182185036955623</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.07090771464597762</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Mo_125Se_400Sb</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Indirect</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>1.03499525750713</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.04085617909626622</v>
+        <v>0.1666805568747302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>